<commit_message>
docs(vault): R0-R2 dual-track scoring, templates, 10 galaxy stubs
- Add source rules, progress tracker, galaxy/profession templates
- Add dual-track scoring (national destiny vs comrade enlistment)
- Add volume weights, license tiers, Excel scoring sheet
- Add V01-V10 thin galaxy notes with protocol anchors
</commit_message>
<xml_diff>
--- a/data/开拓者数据面板_追踪.xlsx
+++ b/data/开拓者数据面板_追踪.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开拓者总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源流水" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蓝图库存" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰队编成" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家国运评分" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="直播开拓币" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="双轨评分说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开拓者总览" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源流水" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蓝图库存" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="舰队编成" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="国家国运评分" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="直播开拓币" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +40,10 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -82,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +107,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,6 +473,348 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>字段/概念</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>对应轨道</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>国运分_卷</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>国家当卷得分=子项加权</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>国运总分</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>各卷国运分×卷权重之和；领袖排序用</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A1协议完成度</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>协议目标交付</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A2控制占有</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>星门/站/矿份额</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A3工业后勤</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>产能维修撤离</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A4军事战果</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>守打而非纯人头</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A5协作秩序</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>团结履约；背刺扣分</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A6文明展示</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>直播组织力；弱权重</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>战友分</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>个人累计(建议衰减累计)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B1岗位胜任</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>本职表现</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>B2危机抗压</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>极限决策</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>B3可协作性</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>混合编队适配</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>B4守序可信度</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>抗腐蚀；一票否决相关</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B5稀缺技能</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>特种不可替代</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B6观察评价</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>人联/高级观众；可关联开拓币但≠国运</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>执照档</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>开拓/对话/勘探/猎人/预备役</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>禁止</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>开拓币直接换国运分；杀敌单极定领袖</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>详设</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>obsidian_vault/10-背景通识/06-考核法与评分/双轨评分逻辑.md</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2049,7 +2397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2383,7 +2731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2627,7 +2975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2837,7 +3185,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5171,7 +5519,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5341,13 +5689,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5427,6 +5775,13 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>10. 本表可与 Obsidian vault 双向链接：人物笔记 frontmatter 的 id 对齐「开拓者ID」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>11. 双轨评分：见 sheet「双轨评分说明」与 vault 双轨评分逻辑.md；国运分国家级，战友分个人级，勿混列。</t>
         </is>
       </c>
     </row>

</xml_diff>